<commit_message>
Rediseno visual estilo Glamour Control + columna Centro de Distribucion en carga Excel
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla-Entradas.xlsx
+++ b/public/plantillas/Plantilla-Entradas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,17 +422,20 @@
       <c r="F1" t="str">
         <v>CANTIDAD KG</v>
       </c>
+      <c r="G1" t="str">
+        <v>CENTRO DE DISTRIBUCION</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -440,6 +443,7 @@
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="34.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,6 +465,9 @@
       <c r="F1" t="str">
         <v>CANTIDAD KG</v>
       </c>
+      <c r="G1" t="str">
+        <v>CENTRO DE DISTRIBUCION</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -481,6 +488,9 @@
       <c r="F2">
         <v>32.5</v>
       </c>
+      <c r="G2" t="str">
+        <v>Lujan</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -501,6 +511,9 @@
       <c r="F3">
         <v>28.14</v>
       </c>
+      <c r="G3" t="str">
+        <v>Campana</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -521,6 +534,9 @@
       <c r="F4">
         <v>36</v>
       </c>
+      <c r="G4" t="str">
+        <v>Campana</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -541,17 +557,20 @@
       <c r="F5">
         <v>21</v>
       </c>
+      <c r="G5" t="str">
+        <v>Lujan</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C38"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -638,31 +657,28 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v xml:space="preserve">  CENTRO DE DISTRIBUCION</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Centro de distribución del movimiento. SOLO: Campana o Lujan. Dejalo vacío si es Lujan.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>UNIDADES POR PRODUCTO (qué número va en CANTIDAD KG):</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">  AF      </v>
-      </c>
-      <c r="B15" t="str">
-        <v xml:space="preserve">ARENA FINA                                   </v>
-      </c>
-      <c r="C15" t="str">
-        <v>tn</v>
+        <v>UNIDADES POR PRODUCTO (qué número va en CANTIDAD KG):</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">  P06     </v>
+        <v xml:space="preserve">  AF      </v>
       </c>
       <c r="B16" t="str">
-        <v xml:space="preserve">PIEDRA 0-6                                   </v>
+        <v xml:space="preserve">ARENA FINA                                   </v>
       </c>
       <c r="C16" t="str">
         <v>tn</v>
@@ -670,10 +686,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">  P612    </v>
+        <v xml:space="preserve">  P06     </v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve">PIEDRA 6-12                                  </v>
+        <v xml:space="preserve">PIEDRA 0-6                                   </v>
       </c>
       <c r="C17" t="str">
         <v>tn</v>
@@ -681,10 +697,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">  P620    </v>
+        <v xml:space="preserve">  P612    </v>
       </c>
       <c r="B18" t="str">
-        <v xml:space="preserve">PIEDRA 6-20                                  </v>
+        <v xml:space="preserve">PIEDRA 6-12                                  </v>
       </c>
       <c r="C18" t="str">
         <v>tn</v>
@@ -692,10 +708,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">  P1030   </v>
+        <v xml:space="preserve">  P620    </v>
       </c>
       <c r="B19" t="str">
-        <v xml:space="preserve">PIEDRA 10-30                                 </v>
+        <v xml:space="preserve">PIEDRA 6-20                                  </v>
       </c>
       <c r="C19" t="str">
         <v>tn</v>
@@ -703,10 +719,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">  E100    </v>
+        <v xml:space="preserve">  P1030   </v>
       </c>
       <c r="B20" t="str">
-        <v xml:space="preserve">ESTABILIZADO 0-100 X TN                      </v>
+        <v xml:space="preserve">PIEDRA 10-30                                 </v>
       </c>
       <c r="C20" t="str">
         <v>tn</v>
@@ -714,10 +730,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v xml:space="preserve">  E020    </v>
+        <v xml:space="preserve">  E100    </v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">ESTABILIZADO GRANULOMETRICO 0/20             </v>
+        <v xml:space="preserve">ESTABILIZADO 0-100 X TN                      </v>
       </c>
       <c r="C21" t="str">
         <v>tn</v>
@@ -725,43 +741,43 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  MS 453  </v>
+        <v xml:space="preserve">  E020    </v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">MIRA SET 453 (ADITIVO)                       </v>
+        <v xml:space="preserve">ESTABILIZADO GRANULOMETRICO 0/20             </v>
       </c>
       <c r="C22" t="str">
-        <v>kg</v>
+        <v>tn</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  C       </v>
+        <v xml:space="preserve">  MS 453  </v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">CPF 40 AVELLANEDA                            </v>
+        <v xml:space="preserve">MIRA SET 453 (ADITIVO)                       </v>
       </c>
       <c r="C23" t="str">
-        <v>tn</v>
+        <v>kg</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  W       </v>
+        <v xml:space="preserve">  C       </v>
       </c>
       <c r="B24" t="str">
-        <v xml:space="preserve">W351R                                        </v>
+        <v xml:space="preserve">CPF 40 AVELLANEDA                            </v>
       </c>
       <c r="C24" t="str">
-        <v>u</v>
+        <v>tn</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  W5      </v>
+        <v xml:space="preserve">  W       </v>
       </c>
       <c r="B25" t="str">
-        <v xml:space="preserve">W500R                                        </v>
+        <v xml:space="preserve">W351R                                        </v>
       </c>
       <c r="C25" t="str">
         <v>u</v>
@@ -769,10 +785,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  S45     </v>
+        <v xml:space="preserve">  W5      </v>
       </c>
       <c r="B26" t="str">
-        <v>SELLADOR (MAPEFLEX PU 45 FT 111 GREY 20X 600ML</v>
+        <v xml:space="preserve">W500R                                        </v>
       </c>
       <c r="C26" t="str">
         <v>u</v>
@@ -780,69 +796,85 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  MFB     </v>
+        <v xml:space="preserve">  S45     </v>
       </c>
       <c r="B27" t="str">
-        <v xml:space="preserve">MAPEFILL E BASGS 25KG                        </v>
+        <v>SELLADOR (MAPEFLEX PU 45 FT 111 GREY 20X 600ML</v>
       </c>
       <c r="C27" t="str">
-        <v>bolsas</v>
+        <v>u</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  RDC     </v>
+        <v xml:space="preserve">  MFB     </v>
       </c>
       <c r="B28" t="str">
-        <v xml:space="preserve">RDC DRUMS 200 KG                             </v>
+        <v xml:space="preserve">MAPEFILL E BASGS 25KG                        </v>
       </c>
       <c r="C28" t="str">
-        <v>tambores</v>
+        <v>bolsas</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v xml:space="preserve">  RDC     </v>
+      </c>
+      <c r="B29" t="str">
+        <v xml:space="preserve">RDC DRUMS 200 KG                             </v>
+      </c>
+      <c r="C29" t="str">
+        <v>tambores</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>REGLAS IMPORTANTES:</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  - No borrar ni renombrar las columnas; no dejar filas vacías entre datos.</v>
+        <v>REGLAS IMPORTANTES:</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  - Cada fila se guarda como un movimiento de tipo ENTRADA de planta Lujan.</v>
+        <v xml:space="preserve">  - No borrar ni renombrar las columnas; no dejar filas vacías entre datos.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  - El sistema ignora automáticamente las filas repetidas (ya cargadas).</v>
+        <v xml:space="preserve">  - CENTRO DE DISTRIBUCION acepta solo "Campana" o "Lujan" (si se deja vacío se carga Lujan).</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  - Si una fila tiene errores, el sistema te avisa antes de importar nada.</v>
+        <v xml:space="preserve">  - Cada fila se guarda como un movimiento de tipo ENTRADA.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v xml:space="preserve">  - El sistema ignora automáticamente las filas repetidas (ya cargadas).</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v xml:space="preserve">  - Si una fila tiene errores, el sistema te avisa antes de importar nada.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
         <v>Ejemplo de carga real de ENTRADAS: ver hoja EJEMPLO (PROVEEDOR + remito + fecha + producto + cantidad).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Plantillas Excel: 3 ejemplos por hoja con datos reales del sistema (centro Lujan)
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla-Entradas.xlsx
+++ b/public/plantillas/Plantilla-Entradas.xlsx
@@ -435,7 +435,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -471,13 +471,13 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2680818</v>
+        <v>105203</v>
       </c>
       <c r="B2" t="str">
         <v>SPOSITO</v>
       </c>
       <c r="C2" s="1">
-        <v>46237</v>
+        <v>46252</v>
       </c>
       <c r="D2" t="str">
         <v>AF</v>
@@ -486,7 +486,7 @@
         <v>ARENA FINA</v>
       </c>
       <c r="F2">
-        <v>32.5</v>
+        <v>35.22</v>
       </c>
       <c r="G2" t="str">
         <v>Lujan</v>
@@ -494,76 +494,53 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>96962</v>
+        <v>110998</v>
       </c>
       <c r="B3" t="str">
-        <v>MESSEL</v>
+        <v>LCE</v>
       </c>
       <c r="C3" s="1">
-        <v>46238</v>
+        <v>46252</v>
       </c>
       <c r="D3" t="str">
-        <v>P620</v>
+        <v>P06</v>
       </c>
       <c r="E3" t="str">
-        <v>PIEDRA 6-20</v>
+        <v>PIEDRA 0-6</v>
       </c>
       <c r="F3">
-        <v>28.14</v>
+        <v>35.06</v>
       </c>
       <c r="G3" t="str">
-        <v>Campana</v>
+        <v>Lujan</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>15755</v>
+        <v>163070</v>
       </c>
       <c r="B4" t="str">
-        <v>CPF AVELLANEDA</v>
+        <v>CA</v>
       </c>
       <c r="C4" s="1">
-        <v>46238</v>
+        <v>46252</v>
       </c>
       <c r="D4" t="str">
-        <v>C</v>
+        <v>P620</v>
       </c>
       <c r="E4" t="str">
-        <v>CPF 40 AVELLANEDA</v>
+        <v>PIEDRA 6-20</v>
       </c>
       <c r="F4">
-        <v>36</v>
+        <v>35.34</v>
       </c>
       <c r="G4" t="str">
-        <v>Campana</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>20411</v>
-      </c>
-      <c r="B5" t="str">
-        <v>SPOSITO</v>
-      </c>
-      <c r="C5" s="1">
-        <v>46239</v>
-      </c>
-      <c r="D5" t="str">
-        <v>MS 453</v>
-      </c>
-      <c r="E5" t="str">
-        <v>MIRA SET 453 (ADITIVO)</v>
-      </c>
-      <c r="F5">
-        <v>21</v>
-      </c>
-      <c r="G5" t="str">
         <v>Lujan</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Plantillas Excel: EJEMPLO como hoja inicial (visible al abrir con los 3 ejemplos)
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla-Entradas.xlsx
+++ b/public/plantillas/Plantilla-Entradas.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="CARGA" sheetId="1" r:id="rId1"/>
-    <sheet name="EJEMPLO" sheetId="2" r:id="rId2"/>
+    <sheet name="EJEMPLO" sheetId="1" r:id="rId1"/>
+    <sheet name="CARGA" sheetId="2" r:id="rId2"/>
     <sheet name="AYUDA" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -401,40 +401,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>REMITOS</v>
-      </c>
-      <c r="B1" t="str">
-        <v>OBSERVACION</v>
-      </c>
-      <c r="C1" t="str">
-        <v>FECHA</v>
-      </c>
-      <c r="D1" t="str">
-        <v>CODIGO DEL PRODUCTO</v>
-      </c>
-      <c r="E1" t="str">
-        <v>DESCRIPCION</v>
-      </c>
-      <c r="F1" t="str">
-        <v>CANTIDAD KG</v>
-      </c>
-      <c r="G1" t="str">
-        <v>CENTRO DE DISTRIBUCION</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -541,6 +507,40 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>REMITOS</v>
+      </c>
+      <c r="B1" t="str">
+        <v>OBSERVACION</v>
+      </c>
+      <c r="C1" t="str">
+        <v>FECHA</v>
+      </c>
+      <c r="D1" t="str">
+        <v>CODIGO DEL PRODUCTO</v>
+      </c>
+      <c r="E1" t="str">
+        <v>DESCRIPCION</v>
+      </c>
+      <c r="F1" t="str">
+        <v>CANTIDAD KG</v>
+      </c>
+      <c r="G1" t="str">
+        <v>CENTRO DE DISTRIBUCION</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Plantillas: CATALOGO visible (sino Excel no muestra el desplegable) + formato de tabla (encabezado azul, filtros, bordes)
</commit_message>
<xml_diff>
--- a/public/plantillas/Plantilla-Entradas.xlsx
+++ b/public/plantillas/Plantilla-Entradas.xlsx
@@ -7,7 +7,7 @@
     <sheet sheetId="1" name="EJEMPLO" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="CARGA" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="AYUDA" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="CATALOGO" state="hidden" r:id="rId7"/>
+    <sheet sheetId="4" name="CATALOGO" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -332,7 +332,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -342,17 +342,28 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3B82F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,17 +371,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -746,78 +775,79 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>105203</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>46252</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="str">
+      <c r="E2" s="2" t="str">
         <f>IFERROR(VLOOKUP($D2,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>35.22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>110998</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>46252</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" t="str">
+      <c r="E3" s="2" t="str">
         <f>IFERROR(VLOOKUP($D3,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>35.06</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>163070</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>46252</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E4" s="2" t="str">
         <f>IFERROR(VLOOKUP($D4,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>35.34</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D4">
       <formula1>'CATALOGO'!$A$2:$A$15</formula1>
@@ -868,601 +898,1196 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E2" t="str">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="str">
         <f>IFERROR(VLOOKUP($D2,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="3" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E3" t="str">
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="str">
         <f>IFERROR(VLOOKUP($D3,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="4" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E4" t="str">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="str">
         <f>IFERROR(VLOOKUP($D4,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="5" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E5" t="str">
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="str">
         <f>IFERROR(VLOOKUP($D5,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="6" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E6" t="str">
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="str">
         <f>IFERROR(VLOOKUP($D6,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="7" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E7" t="str">
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2" t="str">
         <f>IFERROR(VLOOKUP($D7,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E8" t="str">
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2" t="str">
         <f>IFERROR(VLOOKUP($D8,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="9" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E9" t="str">
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="str">
         <f>IFERROR(VLOOKUP($D9,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="10" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E10" t="str">
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="str">
         <f>IFERROR(VLOOKUP($D10,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="11" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E11" t="str">
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="str">
         <f>IFERROR(VLOOKUP($D11,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="12" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E12" t="str">
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2" t="str">
         <f>IFERROR(VLOOKUP($D12,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="13" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E13" t="str">
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2" t="str">
         <f>IFERROR(VLOOKUP($D13,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="14" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E14" t="str">
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2" t="str">
         <f>IFERROR(VLOOKUP($D14,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="15" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E15" t="str">
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2" t="str">
         <f>IFERROR(VLOOKUP($D15,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="16" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E16" t="str">
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2" t="str">
         <f>IFERROR(VLOOKUP($D16,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="17" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E17" t="str">
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2" t="str">
         <f>IFERROR(VLOOKUP($D17,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E18" t="str">
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2" t="str">
         <f>IFERROR(VLOOKUP($D18,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="19" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E19" t="str">
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2" t="str">
         <f>IFERROR(VLOOKUP($D19,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E20" t="str">
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2" t="str">
         <f>IFERROR(VLOOKUP($D20,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E21" t="str">
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2" t="str">
         <f>IFERROR(VLOOKUP($D21,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E22" t="str">
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2" t="str">
         <f>IFERROR(VLOOKUP($D22,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E23" t="str">
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2" t="str">
         <f>IFERROR(VLOOKUP($D23,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E24" t="str">
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2" t="str">
         <f>IFERROR(VLOOKUP($D24,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="25" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E25" t="str">
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2" t="str">
         <f>IFERROR(VLOOKUP($D25,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="26" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E26" t="str">
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2" t="str">
         <f>IFERROR(VLOOKUP($D26,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="27" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E27" t="str">
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2" t="str">
         <f>IFERROR(VLOOKUP($D27,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="28" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E28" t="str">
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2" t="str">
         <f>IFERROR(VLOOKUP($D28,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="29" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E29" t="str">
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2" t="str">
         <f>IFERROR(VLOOKUP($D29,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="30" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E30" t="str">
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2" t="str">
         <f>IFERROR(VLOOKUP($D30,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="31" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E31" t="str">
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2" t="str">
         <f>IFERROR(VLOOKUP($D31,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="32" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E32" t="str">
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2" t="str">
         <f>IFERROR(VLOOKUP($D32,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="33" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E33" t="str">
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2" t="str">
         <f>IFERROR(VLOOKUP($D33,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="34" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E34" t="str">
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2" t="str">
         <f>IFERROR(VLOOKUP($D34,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="35" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E35" t="str">
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2" t="str">
         <f>IFERROR(VLOOKUP($D35,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="36" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E36" t="str">
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2" t="str">
         <f>IFERROR(VLOOKUP($D36,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="37" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E37" t="str">
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2" t="str">
         <f>IFERROR(VLOOKUP($D37,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="38" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E38" t="str">
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2" t="str">
         <f>IFERROR(VLOOKUP($D38,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="39" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E39" t="str">
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2" t="str">
         <f>IFERROR(VLOOKUP($D39,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="40" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E40" t="str">
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2" t="str">
         <f>IFERROR(VLOOKUP($D40,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="41" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E41" t="str">
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2" t="str">
         <f>IFERROR(VLOOKUP($D41,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="42" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E42" t="str">
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2" t="str">
         <f>IFERROR(VLOOKUP($D42,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="43" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E43" t="str">
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2" t="str">
         <f>IFERROR(VLOOKUP($D43,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="44" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E44" t="str">
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2" t="str">
         <f>IFERROR(VLOOKUP($D44,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="45" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E45" t="str">
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2" t="str">
         <f>IFERROR(VLOOKUP($D45,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="46" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E46" t="str">
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2" t="str">
         <f>IFERROR(VLOOKUP($D46,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="47" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E47" t="str">
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2" t="str">
         <f>IFERROR(VLOOKUP($D47,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="48" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E48" t="str">
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2" t="str">
         <f>IFERROR(VLOOKUP($D48,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="49" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E49" t="str">
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2" t="str">
         <f>IFERROR(VLOOKUP($D49,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="50" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E50" t="str">
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2" t="str">
         <f>IFERROR(VLOOKUP($D50,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="51" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E51" t="str">
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2" t="str">
         <f>IFERROR(VLOOKUP($D51,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="52" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E52" t="str">
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2" t="str">
         <f>IFERROR(VLOOKUP($D52,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="53" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E53" t="str">
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2" t="str">
         <f>IFERROR(VLOOKUP($D53,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="54" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E54" t="str">
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2" t="str">
         <f>IFERROR(VLOOKUP($D54,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="55" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E55" t="str">
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2" t="str">
         <f>IFERROR(VLOOKUP($D55,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="56" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E56" t="str">
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2" t="str">
         <f>IFERROR(VLOOKUP($D56,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="57" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E57" t="str">
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2" t="str">
         <f>IFERROR(VLOOKUP($D57,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="58" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E58" t="str">
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2" t="str">
         <f>IFERROR(VLOOKUP($D58,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="59" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E59" t="str">
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2" t="str">
         <f>IFERROR(VLOOKUP($D59,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="60" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E60" t="str">
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2" t="str">
         <f>IFERROR(VLOOKUP($D60,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="61" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E61" t="str">
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2" t="str">
         <f>IFERROR(VLOOKUP($D61,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="62" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E62" t="str">
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2" t="str">
         <f>IFERROR(VLOOKUP($D62,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="63" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E63" t="str">
+      <c r="F62" s="2"/>
+      <c r="G62" s="2"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2" t="str">
         <f>IFERROR(VLOOKUP($D63,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="64" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E64" t="str">
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2" t="str">
         <f>IFERROR(VLOOKUP($D64,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="65" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E65" t="str">
+      <c r="F64" s="2"/>
+      <c r="G64" s="2"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2" t="str">
         <f>IFERROR(VLOOKUP($D65,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="66" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E66" t="str">
+      <c r="F65" s="2"/>
+      <c r="G65" s="2"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2" t="str">
         <f>IFERROR(VLOOKUP($D66,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="67" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E67" t="str">
+      <c r="F66" s="2"/>
+      <c r="G66" s="2"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2" t="str">
         <f>IFERROR(VLOOKUP($D67,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="68" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E68" t="str">
+      <c r="F67" s="2"/>
+      <c r="G67" s="2"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2" t="str">
         <f>IFERROR(VLOOKUP($D68,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="69" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E69" t="str">
+      <c r="F68" s="2"/>
+      <c r="G68" s="2"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2" t="str">
         <f>IFERROR(VLOOKUP($D69,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="70" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E70" t="str">
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="E70" s="2" t="str">
         <f>IFERROR(VLOOKUP($D70,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="71" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E71" t="str">
+      <c r="F70" s="2"/>
+      <c r="G70" s="2"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2" t="str">
         <f>IFERROR(VLOOKUP($D71,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="72" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E72" t="str">
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="2"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
+      <c r="E72" s="2" t="str">
         <f>IFERROR(VLOOKUP($D72,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="73" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E73" t="str">
+      <c r="F72" s="2"/>
+      <c r="G72" s="2"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="2" t="str">
         <f>IFERROR(VLOOKUP($D73,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="74" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E74" t="str">
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2"/>
+      <c r="D74" s="2"/>
+      <c r="E74" s="2" t="str">
         <f>IFERROR(VLOOKUP($D74,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="75" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E75" t="str">
+      <c r="F74" s="2"/>
+      <c r="G74" s="2"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2" t="str">
         <f>IFERROR(VLOOKUP($D75,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="76" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E76" t="str">
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
+      <c r="E76" s="2" t="str">
         <f>IFERROR(VLOOKUP($D76,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="77" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E77" t="str">
+      <c r="F76" s="2"/>
+      <c r="G76" s="2"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" s="2"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
+      <c r="E77" s="2" t="str">
         <f>IFERROR(VLOOKUP($D77,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="78" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E78" t="str">
+      <c r="F77" s="2"/>
+      <c r="G77" s="2"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" s="2"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="E78" s="2" t="str">
         <f>IFERROR(VLOOKUP($D78,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="79" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E79" t="str">
+      <c r="F78" s="2"/>
+      <c r="G78" s="2"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" s="2"/>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2" t="str">
         <f>IFERROR(VLOOKUP($D79,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="80" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E80" t="str">
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="E80" s="2" t="str">
         <f>IFERROR(VLOOKUP($D80,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="81" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E81" t="str">
+      <c r="F80" s="2"/>
+      <c r="G80" s="2"/>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="2"/>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2" t="str">
         <f>IFERROR(VLOOKUP($D81,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="82" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E82" t="str">
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" s="2"/>
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="E82" s="2" t="str">
         <f>IFERROR(VLOOKUP($D82,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="83" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E83" t="str">
+      <c r="F82" s="2"/>
+      <c r="G82" s="2"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2" t="str">
         <f>IFERROR(VLOOKUP($D83,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="84" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E84" t="str">
+      <c r="F83" s="2"/>
+      <c r="G83" s="2"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="E84" s="2" t="str">
         <f>IFERROR(VLOOKUP($D84,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="85" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E85" t="str">
+      <c r="F84" s="2"/>
+      <c r="G84" s="2"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" s="2"/>
+      <c r="B85" s="2"/>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2" t="str">
         <f>IFERROR(VLOOKUP($D85,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="86" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E86" t="str">
+      <c r="F85" s="2"/>
+      <c r="G85" s="2"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="E86" s="2" t="str">
         <f>IFERROR(VLOOKUP($D86,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="87" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E87" t="str">
+      <c r="F86" s="2"/>
+      <c r="G86" s="2"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="E87" s="2" t="str">
         <f>IFERROR(VLOOKUP($D87,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="88" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E88" t="str">
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="2"/>
+      <c r="E88" s="2" t="str">
         <f>IFERROR(VLOOKUP($D88,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="89" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E89" t="str">
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2" t="str">
         <f>IFERROR(VLOOKUP($D89,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="90" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E90" t="str">
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="2"/>
+      <c r="B90" s="2"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="2"/>
+      <c r="E90" s="2" t="str">
         <f>IFERROR(VLOOKUP($D90,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="91" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E91" t="str">
+      <c r="F90" s="2"/>
+      <c r="G90" s="2"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" s="2"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2" t="str">
         <f>IFERROR(VLOOKUP($D91,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="92" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E92" t="str">
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
+      <c r="C92" s="2"/>
+      <c r="D92" s="2"/>
+      <c r="E92" s="2" t="str">
         <f>IFERROR(VLOOKUP($D92,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="93" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E93" t="str">
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2" t="str">
         <f>IFERROR(VLOOKUP($D93,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="94" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E94" t="str">
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
+      <c r="E94" s="2" t="str">
         <f>IFERROR(VLOOKUP($D94,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="95" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E95" t="str">
+      <c r="F94" s="2"/>
+      <c r="G94" s="2"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
+      <c r="E95" s="2" t="str">
         <f>IFERROR(VLOOKUP($D95,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="96" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E96" t="str">
+      <c r="F95" s="2"/>
+      <c r="G95" s="2"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" s="2"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2"/>
+      <c r="E96" s="2" t="str">
         <f>IFERROR(VLOOKUP($D96,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="97" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E97" t="str">
+      <c r="F96" s="2"/>
+      <c r="G96" s="2"/>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" s="2"/>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="E97" s="2" t="str">
         <f>IFERROR(VLOOKUP($D97,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="98" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E98" t="str">
+      <c r="F97" s="2"/>
+      <c r="G97" s="2"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" s="2"/>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2"/>
+      <c r="D98" s="2"/>
+      <c r="E98" s="2" t="str">
         <f>IFERROR(VLOOKUP($D98,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="99" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E99" t="str">
+      <c r="F98" s="2"/>
+      <c r="G98" s="2"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" s="2"/>
+      <c r="B99" s="2"/>
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="E99" s="2" t="str">
         <f>IFERROR(VLOOKUP($D99,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="100" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="E100" t="str">
+      <c r="F99" s="2"/>
+      <c r="G99" s="2"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2" t="str">
         <f>IFERROR(VLOOKUP($D100,'CATALOGO'!$A$2:$B$15,2,FALSE),"")</f>
         <v/>
       </c>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D10:D100">
       <formula1>'CATALOGO'!$A$2:$A$15</formula1>
@@ -1823,14 +2448,14 @@
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1989,6 +2614,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>